<commit_message>
Add Dashboard: full control panel as first sheet
</commit_message>
<xml_diff>
--- a/gta_priority.xlsx
+++ b/gta_priority.xlsx
@@ -7,20 +7,21 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="📋 Все офферы" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="🎬 Монтаж (1 очередь)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="🏆 ТОП Priority" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="💰 ТОП Бюджет" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="🔥 Срочные" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="📄 Полные тексты" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="⚙️ Формула" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="🏠 Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="📋 Все офферы" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="🎬 Монтаж (1 очередь)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="🏆 ТОП Priority" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="💰 ТОП Бюджет" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="🔥 Срочные" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="📄 Полные тексты" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="⚙️ Формула" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'📋 Все офферы'!$A$1:$P$154</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎬 Монтаж (1 очередь)'!$A$1:$P$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'🏆 ТОП Priority'!$A$1:$P$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'💰 ТОП Бюджет'!$A$1:$P$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'🔥 Срочные'!$A$1:$P$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'📋 Все офферы'!$A$1:$P$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'🎬 Монтаж (1 очередь)'!$A$1:$P$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🏆 ТОП Priority'!$A$1:$P$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'💰 ТОП Бюджет'!$A$1:$P$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'🔥 Срочные'!$A$1:$P$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +77,140 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00F0F0EE"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00F0F0EE"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0094A3B8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00378ADD"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005DCAA5"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00F0F0EE"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001D9E75"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00BA7517"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00A32D2D"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007F77DD"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0094A3B8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00F0F0EE"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00378ADD"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005DCAA5"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001D9E75"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00378ADD"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00BA7517"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00378ADD"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001D9E75"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00F0F0EE"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00378ADD"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +241,54 @@
         <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00378ADD"/>
+        <bgColor rgb="00378ADD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001D9E75"/>
+        <bgColor rgb="001D9E75"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BA7517"/>
+        <bgColor rgb="00BA7517"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007F77DD"/>
+        <bgColor rgb="007F77DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00172033"/>
+        <bgColor rgb="00172033"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A32D2D"/>
+        <bgColor rgb="00A32D2D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -135,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -198,6 +379,133 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -560,6 +868,1332 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00378ADD"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="26" t="n"/>
+      <c r="B1" s="26" t="n"/>
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="26" t="n"/>
+      <c r="E1" s="26" t="n"/>
+      <c r="F1" s="26" t="n"/>
+      <c r="G1" s="26" t="n"/>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="26" t="n"/>
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GTA IRL OS — Dashboard</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="n"/>
+      <c r="D2" s="26" t="n"/>
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="26" t="n"/>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Обновлено: 29.06.2026 15:48  ·  Данных: 153 уникальных офферов</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="26" t="n"/>
+      <c r="G3" s="26" t="n"/>
+    </row>
+    <row r="4" ht="8" customHeight="1">
+      <c r="A4" s="26" t="n"/>
+      <c r="B4" s="26" t="n"/>
+      <c r="C4" s="26" t="n"/>
+      <c r="D4" s="26" t="n"/>
+      <c r="E4" s="26" t="n"/>
+      <c r="F4" s="26" t="n"/>
+      <c r="G4" s="26" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  📊  Общая статистика</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="26" t="n"/>
+      <c r="G5" s="26" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Всего найдено офферов</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="n">
+        <v>292</v>
+      </c>
+      <c r="D6" s="26" t="n"/>
+      <c r="E6" s="26" t="n"/>
+      <c r="F6" s="26" t="n"/>
+      <c r="G6" s="26" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Уникальных (без дублей)</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="n">
+        <v>153</v>
+      </c>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="26" t="n"/>
+      <c r="F7" s="26" t="n"/>
+      <c r="G7" s="26" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="26" t="n"/>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Дублей удалено</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>139</v>
+      </c>
+      <c r="D8" s="26" t="n"/>
+      <c r="E8" s="26" t="n"/>
+      <c r="F8" s="26" t="n"/>
+      <c r="G8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="26" t="n"/>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Уникальных заказчиков</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="n">
+        <v>82</v>
+      </c>
+      <c r="D9" s="26" t="n"/>
+      <c r="E9" s="26" t="n"/>
+      <c r="F9" s="26" t="n"/>
+      <c r="G9" s="26" t="n"/>
+    </row>
+    <row r="10" ht="8" customHeight="1">
+      <c r="A10" s="26" t="n"/>
+      <c r="B10" s="26" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="26" t="n"/>
+      <c r="G10" s="26" t="n"/>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="26" t="n"/>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  💰  Денежная статистика</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="26" t="n"/>
+      <c r="E11" s="26" t="n"/>
+      <c r="F11" s="26" t="n"/>
+      <c r="G11" s="26" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="26" t="n"/>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Общий бюджет базы</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="inlineStr">
+        <is>
+          <t>2 149 170 ₽</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="26" t="n"/>
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="26" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="26" t="n"/>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Средний бюджет</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="inlineStr">
+        <is>
+          <t>32 563 ₽</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="26" t="n"/>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Медианный бюджет</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>15 000 ₽</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="n"/>
+      <c r="E14" s="26" t="n"/>
+      <c r="F14" s="26" t="n"/>
+      <c r="G14" s="26" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="26" t="n"/>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Максимальный бюджет</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>120 000 ₽</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="n"/>
+      <c r="E15" s="26" t="n"/>
+      <c r="F15" s="26" t="n"/>
+      <c r="G15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="26" t="n"/>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Минимальный бюджет</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>500 ₽</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="26" t="n"/>
+      <c r="F16" s="26" t="n"/>
+      <c r="G16" s="26" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="26" t="n"/>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Прибыль (сам, 85% маржа)</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>1 826 794 ₽</t>
+        </is>
+      </c>
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="26" t="n"/>
+      <c r="F17" s="26" t="n"/>
+      <c r="G17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="26" t="n"/>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Прибыль (делегировать, 30%)</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>644 751 ₽</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="26" t="n"/>
+      <c r="F18" s="26" t="n"/>
+      <c r="G18" s="26" t="n"/>
+    </row>
+    <row r="19" ht="8" customHeight="1">
+      <c r="A19" s="26" t="n"/>
+      <c r="B19" s="26" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="26" t="n"/>
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="26" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="26" t="n"/>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏱  Время до получения денег</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="26" t="n"/>
+      <c r="F20" s="26" t="n"/>
+      <c r="G20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="26" t="n"/>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Можно закрыть сегодня</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="D21" s="40" t="inlineStr">
+        <is>
+          <t>(срочные заказы)</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="n"/>
+      <c r="F21" s="26" t="n"/>
+      <c r="G21" s="26" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="26" t="n"/>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Можно закрыть за 3 дня</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="40" t="inlineStr">
+        <is>
+          <t>(с дедлайном)</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="26" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="26" t="n"/>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Можно закрыть за неделю</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>(небольшие объёмы)</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="n"/>
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="8" customHeight="1">
+      <c r="A24" s="26" t="n"/>
+      <c r="B24" s="26" t="n"/>
+      <c r="C24" s="26" t="n"/>
+      <c r="D24" s="26" t="n"/>
+      <c r="E24" s="26" t="n"/>
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="26" t="n"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="26" t="n"/>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🎬  Монтаж — первая очередь</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="n"/>
+      <c r="D25" s="26" t="n"/>
+      <c r="E25" s="26" t="n"/>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="26" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="26" t="n"/>
+      <c r="B26" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Найдено заявок по монтажу</t>
+        </is>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="D26" s="26" t="n"/>
+      <c r="E26" s="26" t="n"/>
+      <c r="F26" s="26" t="n"/>
+      <c r="G26" s="26" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="26" t="n"/>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Средний чек</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>45 916 ₽</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="n"/>
+      <c r="E27" s="26" t="n"/>
+      <c r="F27" s="26" t="n"/>
+      <c r="G27" s="26" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="26" t="n"/>
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Потенциальная прибыль (85%)</t>
+        </is>
+      </c>
+      <c r="C28" s="36" t="inlineStr">
+        <is>
+          <t>234 175 ₽</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="n"/>
+      <c r="E28" s="26" t="n"/>
+      <c r="F28" s="26" t="n"/>
+      <c r="G28" s="26" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="26" t="n"/>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Заявок с бюджетом</t>
+        </is>
+      </c>
+      <c r="C29" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="26" t="n"/>
+      <c r="F29" s="26" t="n"/>
+      <c r="G29" s="26" t="n"/>
+    </row>
+    <row r="30" ht="8" customHeight="1">
+      <c r="A30" s="26" t="n"/>
+      <c r="B30" s="26" t="n"/>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="26" t="n"/>
+      <c r="E30" s="26" t="n"/>
+      <c r="F30" s="26" t="n"/>
+      <c r="G30" s="26" t="n"/>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="26" t="n"/>
+      <c r="B31" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🗂  Распределение по нишам</t>
+        </is>
+      </c>
+      <c r="C31" s="26" t="n"/>
+      <c r="D31" s="26" t="n"/>
+      <c r="E31" s="26" t="n"/>
+      <c r="F31" s="26" t="n"/>
+      <c r="G31" s="26" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="26" t="n"/>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t>Ниша</t>
+        </is>
+      </c>
+      <c r="C32" s="45" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="D32" s="45" t="inlineStr">
+        <is>
+          <t>Общий бюджет</t>
+        </is>
+      </c>
+      <c r="E32" s="45" t="inlineStr">
+        <is>
+          <t>Средний чек</t>
+        </is>
+      </c>
+      <c r="F32" s="45" t="inlineStr">
+        <is>
+          <t>Прибыль (85%)</t>
+        </is>
+      </c>
+      <c r="G32" s="26" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="26" t="n"/>
+      <c r="B33" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🎬 монтаж</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>24</v>
+      </c>
+      <c r="D33" s="48" t="inlineStr">
+        <is>
+          <t>275 500 ₽</t>
+        </is>
+      </c>
+      <c r="E33" s="49" t="inlineStr">
+        <is>
+          <t>45 916 ₽</t>
+        </is>
+      </c>
+      <c r="F33" s="50" t="inlineStr">
+        <is>
+          <t>234 175 ₽</t>
+        </is>
+      </c>
+      <c r="G33" s="26" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="26" t="n"/>
+      <c r="B34" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🧠 ai</t>
+        </is>
+      </c>
+      <c r="C34" s="47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" s="48" t="inlineStr">
+        <is>
+          <t>1 600 ₽</t>
+        </is>
+      </c>
+      <c r="E34" s="49" t="inlineStr">
+        <is>
+          <t>800 ₽</t>
+        </is>
+      </c>
+      <c r="F34" s="50" t="inlineStr">
+        <is>
+          <t>1 360 ₽</t>
+        </is>
+      </c>
+      <c r="G34" s="26" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="26" t="n"/>
+      <c r="B35" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🐍 python</t>
+        </is>
+      </c>
+      <c r="C35" s="52" t="n">
+        <v>15</v>
+      </c>
+      <c r="D35" s="53" t="inlineStr">
+        <is>
+          <t>347 000 ₽</t>
+        </is>
+      </c>
+      <c r="E35" s="54" t="inlineStr">
+        <is>
+          <t>38 555 ₽</t>
+        </is>
+      </c>
+      <c r="F35" s="55" t="inlineStr">
+        <is>
+          <t>294 950 ₽</t>
+        </is>
+      </c>
+      <c r="G35" s="26" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="26" t="n"/>
+      <c r="B36" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  📱 smm</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="n">
+        <v>21</v>
+      </c>
+      <c r="D36" s="48" t="inlineStr">
+        <is>
+          <t>396 970 ₽</t>
+        </is>
+      </c>
+      <c r="E36" s="49" t="inlineStr">
+        <is>
+          <t>56 710 ₽</t>
+        </is>
+      </c>
+      <c r="F36" s="50" t="inlineStr">
+        <is>
+          <t>337 424 ₽</t>
+        </is>
+      </c>
+      <c r="G36" s="26" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="26" t="n"/>
+      <c r="B37" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🌐 сайт</t>
+        </is>
+      </c>
+      <c r="C37" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="53" t="inlineStr">
+        <is>
+          <t>40 000 ₽</t>
+        </is>
+      </c>
+      <c r="E37" s="54" t="inlineStr">
+        <is>
+          <t>40 000 ₽</t>
+        </is>
+      </c>
+      <c r="F37" s="55" t="inlineStr">
+        <is>
+          <t>34 000 ₽</t>
+        </is>
+      </c>
+      <c r="G37" s="26" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="26" t="n"/>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🎨 дизайн</t>
+        </is>
+      </c>
+      <c r="C38" s="47" t="n">
+        <v>11</v>
+      </c>
+      <c r="D38" s="48" t="inlineStr">
+        <is>
+          <t>83 000 ₽</t>
+        </is>
+      </c>
+      <c r="E38" s="49" t="inlineStr">
+        <is>
+          <t>27 666 ₽</t>
+        </is>
+      </c>
+      <c r="F38" s="50" t="inlineStr">
+        <is>
+          <t>70 550 ₽</t>
+        </is>
+      </c>
+      <c r="G38" s="26" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="26" t="n"/>
+      <c r="B39" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✍️ копир</t>
+        </is>
+      </c>
+      <c r="C39" s="52" t="n">
+        <v>13</v>
+      </c>
+      <c r="D39" s="53" t="inlineStr">
+        <is>
+          <t>180 000 ₽</t>
+        </is>
+      </c>
+      <c r="E39" s="54" t="inlineStr">
+        <is>
+          <t>15 000 ₽</t>
+        </is>
+      </c>
+      <c r="F39" s="55" t="inlineStr">
+        <is>
+          <t>153 000 ₽</t>
+        </is>
+      </c>
+      <c r="G39" s="26" t="n"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="26" t="n"/>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  📦 другое</t>
+        </is>
+      </c>
+      <c r="C40" s="47" t="n">
+        <v>57</v>
+      </c>
+      <c r="D40" s="48" t="inlineStr">
+        <is>
+          <t>825 100 ₽</t>
+        </is>
+      </c>
+      <c r="E40" s="49" t="inlineStr">
+        <is>
+          <t>31 734 ₽</t>
+        </is>
+      </c>
+      <c r="F40" s="50" t="inlineStr">
+        <is>
+          <t>701 335 ₽</t>
+        </is>
+      </c>
+      <c r="G40" s="26" t="n"/>
+    </row>
+    <row r="41" ht="8" customHeight="1">
+      <c r="A41" s="26" t="n"/>
+      <c r="B41" s="26" t="n"/>
+      <c r="C41" s="26" t="n"/>
+      <c r="D41" s="26" t="n"/>
+      <c r="E41" s="26" t="n"/>
+      <c r="F41" s="26" t="n"/>
+      <c r="G41" s="26" t="n"/>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="26" t="n"/>
+      <c r="B42" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🔄  Воронка продаж</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="n"/>
+      <c r="D42" s="26" t="n"/>
+      <c r="E42" s="26" t="n"/>
+      <c r="F42" s="26" t="n"/>
+      <c r="G42" s="26" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="26" t="n"/>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Найдено</t>
+        </is>
+      </c>
+      <c r="C43" s="56" t="n">
+        <v>292</v>
+      </c>
+      <c r="D43" s="57" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E43" s="26" t="n"/>
+      <c r="F43" s="26" t="n"/>
+      <c r="G43" s="26" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="26" t="n"/>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Уникальных</t>
+        </is>
+      </c>
+      <c r="C44" s="56" t="n">
+        <v>153</v>
+      </c>
+      <c r="D44" s="57" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="E44" s="26" t="n"/>
+      <c r="F44" s="26" t="n"/>
+      <c r="G44" s="26" t="n"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="26" t="n"/>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Отклик отправлен</t>
+        </is>
+      </c>
+      <c r="C45" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="D45" s="57" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="E45" s="26" t="n"/>
+      <c r="F45" s="26" t="n"/>
+      <c r="G45" s="26" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="26" t="n"/>
+      <c r="B46" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Ответили</t>
+        </is>
+      </c>
+      <c r="C46" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="26" t="n"/>
+      <c r="F46" s="26" t="n"/>
+      <c r="G46" s="26" t="n"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="26" t="n"/>
+      <c r="B47" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Переговоры</t>
+        </is>
+      </c>
+      <c r="C47" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="26" t="n"/>
+      <c r="F47" s="26" t="n"/>
+      <c r="G47" s="26" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="26" t="n"/>
+      <c r="B48" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Предоплата</t>
+        </is>
+      </c>
+      <c r="C48" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="n"/>
+      <c r="F48" s="26" t="n"/>
+      <c r="G48" s="26" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="26" t="n"/>
+      <c r="B49" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Закрыто</t>
+        </is>
+      </c>
+      <c r="C49" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="26" t="n"/>
+      <c r="F49" s="26" t="n"/>
+      <c r="G49" s="26" t="n"/>
+    </row>
+    <row r="50" ht="8" customHeight="1">
+      <c r="A50" s="26" t="n"/>
+      <c r="B50" s="26" t="n"/>
+      <c r="C50" s="26" t="n"/>
+      <c r="D50" s="26" t="n"/>
+      <c r="E50" s="26" t="n"/>
+      <c r="F50" s="26" t="n"/>
+      <c r="G50" s="26" t="n"/>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="26" t="n"/>
+      <c r="B51" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🏆  ТОП-10 — открывать прямо сейчас</t>
+        </is>
+      </c>
+      <c r="C51" s="26" t="n"/>
+      <c r="D51" s="26" t="n"/>
+      <c r="E51" s="26" t="n"/>
+      <c r="F51" s="26" t="n"/>
+      <c r="G51" s="26" t="n"/>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="26" t="n"/>
+      <c r="B52" s="45" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C52" s="45" t="inlineStr">
+        <is>
+          <t>Ниша</t>
+        </is>
+      </c>
+      <c r="D52" s="45" t="inlineStr">
+        <is>
+          <t>Контакт</t>
+        </is>
+      </c>
+      <c r="E52" s="45" t="inlineStr">
+        <is>
+          <t>Бюджет</t>
+        </is>
+      </c>
+      <c r="F52" s="45" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="G52" s="26" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="26" t="n"/>
+      <c r="B53" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="53" t="inlineStr">
+        <is>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="D53" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="61" t="inlineStr">
+        <is>
+          <t>60 000₽</t>
+        </is>
+      </c>
+      <c r="F53" s="62" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="G53" s="26" t="n"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="26" t="n"/>
+      <c r="B54" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" s="48" t="inlineStr">
+        <is>
+          <t>монтаж</t>
+        </is>
+      </c>
+      <c r="D54" s="64" t="inlineStr">
+        <is>
+          <t>@busyAssistantXteam</t>
+        </is>
+      </c>
+      <c r="E54" s="65" t="inlineStr">
+        <is>
+          <t>40 000₽</t>
+        </is>
+      </c>
+      <c r="F54" s="66" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G54" s="26" t="n"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="26" t="n"/>
+      <c r="B55" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" s="53" t="inlineStr">
+        <is>
+          <t>монтаж</t>
+        </is>
+      </c>
+      <c r="D55" s="67" t="inlineStr">
+        <is>
+          <t>@aaaaaalbinaa</t>
+        </is>
+      </c>
+      <c r="E55" s="61" t="inlineStr">
+        <is>
+          <t>80 000₽</t>
+        </is>
+      </c>
+      <c r="F55" s="62" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G55" s="26" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="26" t="n"/>
+      <c r="B56" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" s="48" t="inlineStr">
+        <is>
+          <t>прочее</t>
+        </is>
+      </c>
+      <c r="D56" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="65" t="inlineStr">
+        <is>
+          <t>90 000₽</t>
+        </is>
+      </c>
+      <c r="F56" s="66" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="G56" s="26" t="n"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="26" t="n"/>
+      <c r="B57" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" s="53" t="inlineStr">
+        <is>
+          <t>монтаж</t>
+        </is>
+      </c>
+      <c r="D57" s="67" t="inlineStr">
+        <is>
+          <t>@v_grachevsky</t>
+        </is>
+      </c>
+      <c r="E57" s="61" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F57" s="62" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="G57" s="26" t="n"/>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="26" t="n"/>
+      <c r="B58" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="C58" s="48" t="inlineStr">
+        <is>
+          <t>дизайн</t>
+        </is>
+      </c>
+      <c r="D58" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="65" t="inlineStr">
+        <is>
+          <t>50 000₽</t>
+        </is>
+      </c>
+      <c r="F58" s="66" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G58" s="26" t="n"/>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="26" t="n"/>
+      <c r="B59" s="59" t="n">
+        <v>7</v>
+      </c>
+      <c r="C59" s="53" t="inlineStr">
+        <is>
+          <t>дизайн</t>
+        </is>
+      </c>
+      <c r="D59" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="61" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F59" s="62" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="G59" s="26" t="n"/>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="26" t="n"/>
+      <c r="B60" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="C60" s="48" t="inlineStr">
+        <is>
+          <t>монтаж</t>
+        </is>
+      </c>
+      <c r="D60" s="68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="65" t="inlineStr">
+        <is>
+          <t>50 000₽</t>
+        </is>
+      </c>
+      <c r="F60" s="66" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="G60" s="26" t="n"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="26" t="n"/>
+      <c r="B61" s="59" t="n">
+        <v>9</v>
+      </c>
+      <c r="C61" s="53" t="inlineStr">
+        <is>
+          <t>монтаж</t>
+        </is>
+      </c>
+      <c r="D61" s="67" t="inlineStr">
+        <is>
+          <t>@Filippova_Anya</t>
+        </is>
+      </c>
+      <c r="E61" s="61" t="inlineStr">
+        <is>
+          <t>60 000₽</t>
+        </is>
+      </c>
+      <c r="F61" s="62" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="G61" s="26" t="n"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="26" t="n"/>
+      <c r="B62" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="C62" s="48" t="inlineStr">
+        <is>
+          <t>монтаж</t>
+        </is>
+      </c>
+      <c r="D62" s="64" t="inlineStr">
+        <is>
+          <t>@Myach_kvadrat</t>
+        </is>
+      </c>
+      <c r="E62" s="65" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F62" s="66" t="n">
+        <v>6</v>
+      </c>
+      <c r="G62" s="26" t="n"/>
+    </row>
+    <row r="63" ht="8" customHeight="1">
+      <c r="A63" s="26" t="n"/>
+      <c r="B63" s="26" t="n"/>
+      <c r="C63" s="26" t="n"/>
+      <c r="D63" s="26" t="n"/>
+      <c r="E63" s="26" t="n"/>
+      <c r="F63" s="26" t="n"/>
+      <c r="G63" s="26" t="n"/>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="26" t="n"/>
+      <c r="B64" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🤖  AI &amp; Эффективность</t>
+        </is>
+      </c>
+      <c r="C64" s="26" t="n"/>
+      <c r="D64" s="26" t="n"/>
+      <c r="E64" s="26" t="n"/>
+      <c r="F64" s="26" t="n"/>
+      <c r="G64" s="26" t="n"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="26" t="n"/>
+      <c r="B65" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Обработано без AI (rule-based)</t>
+        </is>
+      </c>
+      <c r="C65" s="36" t="inlineStr">
+        <is>
+          <t>153 из 153</t>
+        </is>
+      </c>
+      <c r="D65" s="40" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="n"/>
+      <c r="F65" s="26" t="n"/>
+      <c r="G65" s="26" t="n"/>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="26" t="n"/>
+      <c r="B66" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AI-запросов на анализ</t>
+        </is>
+      </c>
+      <c r="C66" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="40" t="inlineStr">
+        <is>
+          <t>(скоринг rule-based)</t>
+        </is>
+      </c>
+      <c r="E66" s="26" t="n"/>
+      <c r="F66" s="26" t="n"/>
+      <c r="G66" s="26" t="n"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="26" t="n"/>
+      <c r="B67" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Стоимость анализа 1 заявки</t>
+        </is>
+      </c>
+      <c r="C67" s="36" t="inlineStr">
+        <is>
+          <t>0₽</t>
+        </is>
+      </c>
+      <c r="D67" s="40" t="inlineStr">
+        <is>
+          <t>(нет расхода токенов)</t>
+        </is>
+      </c>
+      <c r="E67" s="26" t="n"/>
+      <c r="F67" s="26" t="n"/>
+      <c r="G67" s="26" t="n"/>
+    </row>
+    <row r="68" ht="8" customHeight="1">
+      <c r="A68" s="26" t="n"/>
+      <c r="B68" s="26" t="n"/>
+      <c r="C68" s="26" t="n"/>
+      <c r="D68" s="26" t="n"/>
+      <c r="E68" s="26" t="n"/>
+      <c r="F68" s="26" t="n"/>
+      <c r="G68" s="26" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="26" t="n"/>
+      <c r="B69" s="26" t="n"/>
+      <c r="C69" s="26" t="n"/>
+      <c r="D69" s="26" t="n"/>
+      <c r="E69" s="26" t="n"/>
+      <c r="F69" s="26" t="n"/>
+      <c r="G69" s="26" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="26" t="n"/>
+      <c r="B70" s="26" t="n"/>
+      <c r="C70" s="26" t="n"/>
+      <c r="D70" s="26" t="n"/>
+      <c r="E70" s="26" t="n"/>
+      <c r="F70" s="26" t="n"/>
+      <c r="G70" s="26" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="26" t="n"/>
+      <c r="B71" s="26" t="n"/>
+      <c r="C71" s="26" t="n"/>
+      <c r="D71" s="26" t="n"/>
+      <c r="E71" s="26" t="n"/>
+      <c r="F71" s="26" t="n"/>
+      <c r="G71" s="26" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="26" t="n"/>
+      <c r="B72" s="26" t="n"/>
+      <c r="C72" s="26" t="n"/>
+      <c r="D72" s="26" t="n"/>
+      <c r="E72" s="26" t="n"/>
+      <c r="F72" s="26" t="n"/>
+      <c r="G72" s="26" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="26" t="n"/>
+      <c r="B73" s="26" t="n"/>
+      <c r="C73" s="26" t="n"/>
+      <c r="D73" s="26" t="n"/>
+      <c r="E73" s="26" t="n"/>
+      <c r="F73" s="26" t="n"/>
+      <c r="G73" s="26" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="B31:F31"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId5"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -12245,7 +13879,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14256,7 +15890,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18199,7 +19833,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21404,7 +23038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23622,7 +25256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27593,7 +29227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>